<commit_message>
up to july 2026
</commit_message>
<xml_diff>
--- a/final_run_2026/all_subj_methods_anova/cost_lvl_comparisons.xlsx
+++ b/final_run_2026/all_subj_methods_anova/cost_lvl_comparisons.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="5384" uniqueCount="4207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="10066" uniqueCount="4343">
   <si>
     <t>subject level observations</t>
   </si>
@@ -12642,6 +12642,414 @@
   </si>
   <si>
     <t>0.032082</t>
+  </si>
+  <si>
+    <t>52.9618</t>
+  </si>
+  <si>
+    <t>55.4167</t>
+  </si>
+  <si>
+    <t>53.7325</t>
+  </si>
+  <si>
+    <t>66.534</t>
+  </si>
+  <si>
+    <t>63.553</t>
+  </si>
+  <si>
+    <t>51.3084</t>
+  </si>
+  <si>
+    <t>52.1546</t>
+  </si>
+  <si>
+    <t>44.3497</t>
+  </si>
+  <si>
+    <t>41.5424</t>
+  </si>
+  <si>
+    <t>46.9016</t>
+  </si>
+  <si>
+    <t>57.3083</t>
+  </si>
+  <si>
+    <t>55.1504</t>
+  </si>
+  <si>
+    <t>54.0125</t>
+  </si>
+  <si>
+    <t>38.268</t>
+  </si>
+  <si>
+    <t>38.9301</t>
+  </si>
+  <si>
+    <t>37.6111</t>
+  </si>
+  <si>
+    <t>41.8537</t>
+  </si>
+  <si>
+    <t>25.375</t>
+  </si>
+  <si>
+    <t>56.7578</t>
+  </si>
+  <si>
+    <t>31.8222</t>
+  </si>
+  <si>
+    <t>44.9565</t>
+  </si>
+  <si>
+    <t>37.1143</t>
+  </si>
+  <si>
+    <t>35.6348</t>
+  </si>
+  <si>
+    <t>24.3333</t>
+  </si>
+  <si>
+    <t>47.2857</t>
+  </si>
+  <si>
+    <t>32.2925</t>
+  </si>
+  <si>
+    <t>29.6977</t>
+  </si>
+  <si>
+    <t>1.2563</t>
+  </si>
+  <si>
+    <t>1.4005</t>
+  </si>
+  <si>
+    <t>1.6467</t>
+  </si>
+  <si>
+    <t>1.4369</t>
+  </si>
+  <si>
+    <t>1.5461</t>
+  </si>
+  <si>
+    <t>1.7107</t>
+  </si>
+  <si>
+    <t>1.2982</t>
+  </si>
+  <si>
+    <t>1.4945</t>
+  </si>
+  <si>
+    <t>1.5782</t>
+  </si>
+  <si>
+    <t>1.4941</t>
+  </si>
+  <si>
+    <t>1.7804</t>
+  </si>
+  <si>
+    <t>1.5236</t>
+  </si>
+  <si>
+    <t>1.2406</t>
+  </si>
+  <si>
+    <t>1.4335</t>
+  </si>
+  <si>
+    <t>1.6665</t>
+  </si>
+  <si>
+    <t>1.37</t>
+  </si>
+  <si>
+    <t>1.5626</t>
+  </si>
+  <si>
+    <t>1.6743</t>
+  </si>
+  <si>
+    <t>1.2818</t>
+  </si>
+  <si>
+    <t>1.5152</t>
+  </si>
+  <si>
+    <t>1.6468</t>
+  </si>
+  <si>
+    <t>1.2659</t>
+  </si>
+  <si>
+    <t>1.5995</t>
+  </si>
+  <si>
+    <t>1.5402</t>
+  </si>
+  <si>
+    <t>1.6569</t>
+  </si>
+  <si>
+    <t>2.9344</t>
+  </si>
+  <si>
+    <t>3.1885</t>
+  </si>
+  <si>
+    <t>2.9433</t>
+  </si>
+  <si>
+    <t>2.8574</t>
+  </si>
+  <si>
+    <t>2.9099</t>
+  </si>
+  <si>
+    <t>2.7039</t>
+  </si>
+  <si>
+    <t>2.747</t>
+  </si>
+  <si>
+    <t>2.9488</t>
+  </si>
+  <si>
+    <t>3.1346</t>
+  </si>
+  <si>
+    <t>2.9216</t>
+  </si>
+  <si>
+    <t>2.9161</t>
+  </si>
+  <si>
+    <t>2.6901</t>
+  </si>
+  <si>
+    <t>3.1404</t>
+  </si>
+  <si>
+    <t>2.7719</t>
+  </si>
+  <si>
+    <t>2.9555</t>
+  </si>
+  <si>
+    <t>3.1721</t>
+  </si>
+  <si>
+    <t>2.9506</t>
+  </si>
+  <si>
+    <t>2.834</t>
+  </si>
+  <si>
+    <t>2.9529</t>
+  </si>
+  <si>
+    <t>2.7171</t>
+  </si>
+  <si>
+    <t>2.7665</t>
+  </si>
+  <si>
+    <t>2.9463</t>
+  </si>
+  <si>
+    <t>3.1544</t>
+  </si>
+  <si>
+    <t>2.9166</t>
+  </si>
+  <si>
+    <t>2.8444</t>
+  </si>
+  <si>
+    <t>2.9175</t>
+  </si>
+  <si>
+    <t>2.7003</t>
+  </si>
+  <si>
+    <t>3.1025</t>
+  </si>
+  <si>
+    <t>2.7759</t>
+  </si>
+  <si>
+    <t>171.4107</t>
+  </si>
+  <si>
+    <t>259.5932</t>
+  </si>
+  <si>
+    <t>180.2042</t>
+  </si>
+  <si>
+    <t>151.9612</t>
+  </si>
+  <si>
+    <t>295.1508</t>
+  </si>
+  <si>
+    <t>318.76</t>
+  </si>
+  <si>
+    <t>273.7708</t>
+  </si>
+  <si>
+    <t>139.88</t>
+  </si>
+  <si>
+    <t>241.8814</t>
+  </si>
+  <si>
+    <t>193.4091</t>
+  </si>
+  <si>
+    <t>430.1825</t>
+  </si>
+  <si>
+    <t>290.0367</t>
+  </si>
+  <si>
+    <t>271.9125</t>
+  </si>
+  <si>
+    <t>301.8454</t>
+  </si>
+  <si>
+    <t>155.39706</t>
+  </si>
+  <si>
+    <t>233.77778</t>
+  </si>
+  <si>
+    <t>196.48598</t>
+  </si>
+  <si>
+    <t>138.71875</t>
+  </si>
+  <si>
+    <t>377.73387</t>
+  </si>
+  <si>
+    <t>340.18293</t>
+  </si>
+  <si>
+    <t>379.1413</t>
+  </si>
+  <si>
+    <t>174.80769</t>
+  </si>
+  <si>
+    <t>237.2381</t>
+  </si>
+  <si>
+    <t>169.92929</t>
+  </si>
+  <si>
+    <t>114.31429</t>
+  </si>
+  <si>
+    <t>353.37037</t>
+  </si>
+  <si>
+    <t>243.81132</t>
+  </si>
+  <si>
+    <t>286.93023</t>
+  </si>
+  <si>
+    <t>305.0495</t>
+  </si>
+  <si>
+    <t>1.4821</t>
+  </si>
+  <si>
+    <t>2.6271</t>
+  </si>
+  <si>
+    <t>1.8239</t>
+  </si>
+  <si>
+    <t>2.373</t>
+  </si>
+  <si>
+    <t>2.14</t>
+  </si>
+  <si>
+    <t>2.4167</t>
+  </si>
+  <si>
+    <t>1.424</t>
+  </si>
+  <si>
+    <t>2.2881</t>
+  </si>
+  <si>
+    <t>2.0909</t>
+  </si>
+  <si>
+    <t>2.6032</t>
+  </si>
+  <si>
+    <t>2.3211</t>
+  </si>
+  <si>
+    <t>2.2784</t>
+  </si>
+  <si>
+    <t>1.4779</t>
+  </si>
+  <si>
+    <t>1.8519</t>
+  </si>
+  <si>
+    <t>1.9252</t>
+  </si>
+  <si>
+    <t>1.8125</t>
+  </si>
+  <si>
+    <t>3.0806</t>
+  </si>
+  <si>
+    <t>2.5854</t>
+  </si>
+  <si>
+    <t>1.8769</t>
+  </si>
+  <si>
+    <t>2.3968</t>
+  </si>
+  <si>
+    <t>1.8485</t>
+  </si>
+  <si>
+    <t>1.6381</t>
+  </si>
+  <si>
+    <t>2.1759</t>
+  </si>
+  <si>
+    <t>1.9811</t>
+  </si>
+  <si>
+    <t>2.6279</t>
+  </si>
+  <si>
+    <t>2.2079</t>
   </si>
 </sst>
 </file>
@@ -12763,7 +13171,7 @@
         <v>848</v>
       </c>
       <c r="H2" s="0">
-        <v>75807.612890898105</v>
+        <v>75825.020331210777</v>
       </c>
       <c r="I2" s="0">
         <v>3</v>
@@ -12772,13 +13180,13 @@
         <v>0</v>
       </c>
       <c r="K2" s="0">
-        <v>25269.204296966036</v>
+        <v>25275.006777070259</v>
       </c>
       <c r="L2" s="0">
-        <v>70.252053334486376</v>
+        <v>70.239237428273285</v>
       </c>
       <c r="M2" s="0">
-        <v>3.8968032035630793e-41</v>
+        <v>3.9585968718532294e-41</v>
       </c>
       <c r="O2" s="0" t="s">
         <v>868</v>
@@ -12801,7 +13209,7 @@
         <v>849</v>
       </c>
       <c r="H3" s="0">
-        <v>350701.125734178</v>
+        <v>350845.65991777042</v>
       </c>
       <c r="I3" s="0">
         <v>975</v>
@@ -12810,7 +13218,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="0">
-        <v>359.69346229146464</v>
+        <v>359.84170247976454</v>
       </c>
       <c r="L3" s="0"/>
       <c r="M3" s="0"/>
@@ -12820,22 +13228,22 @@
     </row>
     <row r="4">
       <c r="B4" s="0" t="s">
-        <v>4</v>
+        <v>4207</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>234</v>
+        <v>4214</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>447</v>
+        <v>4221</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>652</v>
+        <v>4228</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>850</v>
       </c>
       <c r="H4" s="0">
-        <v>426508.73862507613</v>
+        <v>426670.68024898123</v>
       </c>
       <c r="I4" s="0">
         <v>978</v>
@@ -12966,16 +13374,16 @@
         <v>859</v>
       </c>
       <c r="I11" s="0">
-        <v>-1.7036866028083661</v>
+        <v>-1.7234284986066166</v>
       </c>
       <c r="J11" s="0">
-        <v>2.6940164189657523</v>
+        <v>2.6751806407895415</v>
       </c>
       <c r="K11" s="0">
-        <v>7.0917194407398707</v>
+        <v>7.0737897801856997</v>
       </c>
       <c r="L11" s="0">
-        <v>0.39366415395992149</v>
+        <v>0.40026364705002804</v>
       </c>
     </row>
     <row r="12">
@@ -12998,13 +13406,13 @@
         <v>860</v>
       </c>
       <c r="I12" s="0">
-        <v>12.442894836397086</v>
+        <v>12.423588311124298</v>
       </c>
       <c r="J12" s="0">
-        <v>16.84511056294447</v>
+        <v>16.826711085106695</v>
       </c>
       <c r="K12" s="0">
-        <v>21.247326289491852</v>
+        <v>21.229833859089091</v>
       </c>
       <c r="L12" s="0">
         <v>2.5626123979254146e-23</v>
@@ -13030,13 +13438,13 @@
         <v>862</v>
       </c>
       <c r="I13" s="0">
-        <v>16.058124734179433</v>
+        <v>16.059533374975814</v>
       </c>
       <c r="J13" s="0">
-        <v>20.460340460726819</v>
+        <v>20.46265614895821</v>
       </c>
       <c r="K13" s="0">
-        <v>24.862556187274205</v>
+        <v>24.865778922940606</v>
       </c>
       <c r="L13" s="0">
         <v>0</v>
@@ -13062,16 +13470,16 @@
         <v>860</v>
       </c>
       <c r="I14" s="0">
-        <v>9.744406966381117</v>
+        <v>9.7439352979716247</v>
       </c>
       <c r="J14" s="0">
-        <v>14.151094143978717</v>
+        <v>14.151530444317153</v>
       </c>
       <c r="K14" s="0">
-        <v>18.557781321576318</v>
+        <v>18.559125590662681</v>
       </c>
       <c r="L14" s="0">
-        <v>5.0944180750918147e-16</v>
+        <v>5.1611618006740549e-16</v>
       </c>
     </row>
     <row r="15">
@@ -13094,13 +13502,13 @@
         <v>862</v>
       </c>
       <c r="I15" s="0">
-        <v>13.359636864163466</v>
+        <v>13.37988036182314</v>
       </c>
       <c r="J15" s="0">
-        <v>17.766324041761067</v>
+        <v>17.787475508168669</v>
       </c>
       <c r="K15" s="0">
-        <v>22.173011219358667</v>
+        <v>22.195070654514197</v>
       </c>
       <c r="L15" s="0">
         <v>0</v>
@@ -13126,16 +13534,16 @@
         <v>862</v>
       </c>
       <c r="I16" s="0">
-        <v>-0.79596079369120787</v>
+        <v>-0.77615452428921827</v>
       </c>
       <c r="J16" s="0">
-        <v>3.6152298977823492</v>
+        <v>3.6359450638515156</v>
       </c>
       <c r="K16" s="0">
-        <v>8.0264205892559062</v>
+        <v>8.0480446519922495</v>
       </c>
       <c r="L16" s="0">
-        <v>0.15128718807616159</v>
+        <v>0.14759481414979103</v>
       </c>
     </row>
     <row r="17">
@@ -13280,16 +13688,16 @@
     </row>
     <row r="27">
       <c r="B27" s="0" t="s">
-        <v>26</v>
+        <v>4208</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>254</v>
+        <v>4215</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>465</v>
+        <v>4222</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>335</v>
+        <v>169</v>
       </c>
     </row>
     <row r="28">
@@ -13650,16 +14058,16 @@
     </row>
     <row r="54">
       <c r="B54" s="0" t="s">
-        <v>51</v>
+        <v>4209</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>278</v>
+        <v>4216</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>486</v>
+        <v>4223</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>343</v>
+        <v>4229</v>
       </c>
     </row>
     <row r="55">
@@ -13748,16 +14156,16 @@
     </row>
     <row r="61">
       <c r="B61" s="0" t="s">
-        <v>57</v>
+        <v>4210</v>
       </c>
       <c r="C61" s="0" t="s">
         <v>285</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>492</v>
+        <v>4224</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>695</v>
+        <v>4230</v>
       </c>
     </row>
     <row r="62">
@@ -15512,16 +15920,16 @@
     </row>
     <row r="189">
       <c r="B189" s="0" t="s">
-        <v>175</v>
+        <v>4211</v>
       </c>
       <c r="C189" s="0" t="s">
-        <v>389</v>
+        <v>4217</v>
       </c>
       <c r="D189" s="0" t="s">
-        <v>595</v>
+        <v>4225</v>
       </c>
       <c r="E189" s="0" t="s">
-        <v>796</v>
+        <v>4231</v>
       </c>
     </row>
     <row r="190">
@@ -15610,16 +16018,16 @@
     </row>
     <row r="196">
       <c r="B196" s="0" t="s">
-        <v>182</v>
+        <v>4212</v>
       </c>
       <c r="C196" s="0" t="s">
-        <v>396</v>
+        <v>4218</v>
       </c>
       <c r="D196" s="0" t="s">
-        <v>602</v>
+        <v>4226</v>
       </c>
       <c r="E196" s="0" t="s">
-        <v>802</v>
+        <v>4232</v>
       </c>
     </row>
     <row r="197">
@@ -16061,13 +16469,13 @@
         <v>210</v>
       </c>
       <c r="C228" s="0" t="s">
-        <v>426</v>
+        <v>4219</v>
       </c>
       <c r="D228" s="0" t="s">
         <v>630</v>
       </c>
       <c r="E228" s="0" t="s">
-        <v>827</v>
+        <v>4233</v>
       </c>
     </row>
     <row r="229">
@@ -16338,16 +16746,16 @@
     </row>
     <row r="248">
       <c r="B248" s="0" t="s">
-        <v>229</v>
+        <v>4213</v>
       </c>
       <c r="C248" s="0" t="s">
-        <v>441</v>
+        <v>4220</v>
       </c>
       <c r="D248" s="0" t="s">
-        <v>646</v>
+        <v>4227</v>
       </c>
       <c r="E248" s="0" t="s">
-        <v>844</v>
+        <v>515</v>
       </c>
     </row>
     <row r="249">
@@ -16466,7 +16874,7 @@
         <v>848</v>
       </c>
       <c r="H2" s="0">
-        <v>0.13997439905299147</v>
+        <v>0.13698803455355288</v>
       </c>
       <c r="I2" s="0">
         <v>3</v>
@@ -16475,13 +16883,13 @@
         <v>0</v>
       </c>
       <c r="K2" s="0">
-        <v>0.046658133017663826</v>
+        <v>0.045662678184517629</v>
       </c>
       <c r="L2" s="0">
-        <v>0.52635307606581871</v>
+        <v>0.51561315542358488</v>
       </c>
       <c r="M2" s="0">
-        <v>0.66428537286506684</v>
+        <v>0.67163126687260322</v>
       </c>
       <c r="O2" s="0" t="s">
         <v>868</v>
@@ -16504,7 +16912,7 @@
         <v>849</v>
       </c>
       <c r="H3" s="0">
-        <v>66.749062102769059</v>
+        <v>66.685646615619689</v>
       </c>
       <c r="I3" s="0">
         <v>753</v>
@@ -16513,7 +16921,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="0">
-        <v>0.088644172779241776</v>
+        <v>0.088559955664833587</v>
       </c>
       <c r="L3" s="0"/>
       <c r="M3" s="0"/>
@@ -16523,22 +16931,22 @@
     </row>
     <row r="4">
       <c r="B4" s="0" t="s">
-        <v>872</v>
+        <v>1156</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>1063</v>
+        <v>4239</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>1241</v>
+        <v>4245</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>1421</v>
+        <v>3175</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>850</v>
       </c>
       <c r="H4" s="0">
-        <v>66.889036501822048</v>
+        <v>66.822634650173242</v>
       </c>
       <c r="I4" s="0">
         <v>756</v>
@@ -16645,16 +17053,16 @@
         <v>859</v>
       </c>
       <c r="I11" s="0">
-        <v>-0.053874884929489247</v>
+        <v>-0.054275507715374025</v>
       </c>
       <c r="J11" s="0">
-        <v>0.024835256862732136</v>
+        <v>0.024397235588152988</v>
       </c>
       <c r="K11" s="0">
-        <v>0.10354539865495352</v>
+        <v>0.10306997889168</v>
       </c>
       <c r="L11" s="0">
-        <v>0.84949592886286773</v>
+        <v>0.85597526765792964</v>
       </c>
     </row>
     <row r="12">
@@ -16677,16 +17085,16 @@
         <v>860</v>
       </c>
       <c r="I12" s="0">
-        <v>-0.080257588110938291</v>
+        <v>-0.080711413835058962</v>
       </c>
       <c r="J12" s="0">
-        <v>-0.0023935820225233773</v>
+        <v>-0.0028844042007869497</v>
       </c>
       <c r="K12" s="0">
-        <v>0.075470424065891537</v>
+        <v>0.074942605433485063</v>
       </c>
       <c r="L12" s="0">
-        <v>0.99982350105161477</v>
+        <v>0.99969102711439217</v>
       </c>
     </row>
     <row r="13">
@@ -16709,16 +17117,16 @@
         <v>862</v>
       </c>
       <c r="I13" s="0">
-        <v>-0.090942484911371746</v>
+        <v>-0.090852381193316456</v>
       </c>
       <c r="J13" s="0">
-        <v>-0.012557046642824199</v>
+        <v>-0.012504187133204336</v>
       </c>
       <c r="K13" s="0">
-        <v>0.065828391625723348</v>
+        <v>0.065844006926907783</v>
       </c>
       <c r="L13" s="0">
-        <v>0.97649424853492828</v>
+        <v>0.97674586710836564</v>
       </c>
     </row>
     <row r="14">
@@ -16735,16 +17143,16 @@
         <v>860</v>
       </c>
       <c r="I14" s="0">
-        <v>-0.10613828008400851</v>
+        <v>-0.10615358780349385</v>
       </c>
       <c r="J14" s="0">
-        <v>-0.027228838885255513</v>
+        <v>-0.027281639788939938</v>
       </c>
       <c r="K14" s="0">
-        <v>0.051680602313497484</v>
+        <v>0.051590308225613973</v>
       </c>
       <c r="L14" s="0">
-        <v>0.81190343489767203</v>
+        <v>0.81078988705549293</v>
       </c>
     </row>
     <row r="15">
@@ -16767,16 +17175,16 @@
         <v>862</v>
       </c>
       <c r="I15" s="0">
-        <v>-0.11681631372107631</v>
+        <v>-0.11628769525936239</v>
       </c>
       <c r="J15" s="0">
-        <v>-0.037392303505556335</v>
+        <v>-0.036901422721357324</v>
       </c>
       <c r="K15" s="0">
-        <v>0.042031706709963645</v>
+        <v>0.042484849816647741</v>
       </c>
       <c r="L15" s="0">
-        <v>0.62079321982868141</v>
+        <v>0.63053178407492327</v>
       </c>
     </row>
     <row r="16">
@@ -16799,16 +17207,16 @@
         <v>862</v>
       </c>
       <c r="I16" s="0">
-        <v>-0.088749025774371229</v>
+        <v>-0.088168004791278287</v>
       </c>
       <c r="J16" s="0">
-        <v>-0.010163464620300822</v>
+        <v>-0.0096197829324173867</v>
       </c>
       <c r="K16" s="0">
-        <v>0.068422096533769586</v>
+        <v>0.068928438926443514</v>
       </c>
       <c r="L16" s="0">
-        <v>0.9873581018018055</v>
+        <v>0.98921939739917475</v>
       </c>
     </row>
     <row r="17">
@@ -16937,16 +17345,16 @@
     </row>
     <row r="27">
       <c r="B27" s="0" t="s">
-        <v>889</v>
+        <v>4234</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>1078</v>
+        <v>4240</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>1258</v>
+        <v>4246</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>1436</v>
+        <v>4252</v>
       </c>
     </row>
     <row r="28">
@@ -17281,16 +17689,16 @@
     </row>
     <row r="54">
       <c r="B54" s="0" t="s">
-        <v>912</v>
+        <v>4235</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>1099</v>
+        <v>4241</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>1281</v>
+        <v>4247</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>1457</v>
+        <v>4253</v>
       </c>
     </row>
     <row r="55">
@@ -17379,16 +17787,16 @@
     </row>
     <row r="61">
       <c r="B61" s="0" t="s">
-        <v>919</v>
+        <v>4236</v>
       </c>
       <c r="C61" s="0" t="s">
         <v>1106</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>1288</v>
+        <v>4248</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>1463</v>
+        <v>4254</v>
       </c>
     </row>
     <row r="62">
@@ -18865,16 +19273,16 @@
     </row>
     <row r="189">
       <c r="B189" s="0" t="s">
-        <v>1012</v>
+        <v>4237</v>
       </c>
       <c r="C189" s="0" t="s">
-        <v>1191</v>
+        <v>1458</v>
       </c>
       <c r="D189" s="0" t="s">
-        <v>1370</v>
+        <v>4249</v>
       </c>
       <c r="E189" s="0" t="s">
-        <v>1543</v>
+        <v>4255</v>
       </c>
     </row>
     <row r="190">
@@ -18955,16 +19363,16 @@
     </row>
     <row r="196">
       <c r="B196" s="0" t="s">
-        <v>1018</v>
+        <v>4238</v>
       </c>
       <c r="C196" s="0" t="s">
-        <v>1197</v>
+        <v>4242</v>
       </c>
       <c r="D196" s="0" t="s">
-        <v>1375</v>
+        <v>4250</v>
       </c>
       <c r="E196" s="0" t="s">
-        <v>1549</v>
+        <v>4256</v>
       </c>
     </row>
     <row r="197">
@@ -19382,13 +19790,13 @@
         <v>1045</v>
       </c>
       <c r="C228" s="0" t="s">
-        <v>1223</v>
+        <v>4243</v>
       </c>
       <c r="D228" s="0" t="s">
         <v>1402</v>
       </c>
       <c r="E228" s="0" t="s">
-        <v>1577</v>
+        <v>4257</v>
       </c>
     </row>
     <row r="229">
@@ -19621,16 +20029,16 @@
     </row>
     <row r="248">
       <c r="B248" s="0" t="s">
-        <v>1060</v>
+        <v>3195</v>
       </c>
       <c r="C248" s="0" t="s">
-        <v>1238</v>
+        <v>4244</v>
       </c>
       <c r="D248" s="0" t="s">
-        <v>1418</v>
+        <v>4251</v>
       </c>
       <c r="E248" s="0" t="s">
-        <v>1592</v>
+        <v>4258</v>
       </c>
     </row>
     <row r="249">
@@ -19679,7 +20087,7 @@
     <col min="10" max="10" width="15.21875" customWidth="true"/>
     <col min="11" max="11" width="13.5546875" customWidth="true"/>
     <col min="12" max="12" width="12.5546875" customWidth="true"/>
-    <col min="13" max="13" width="12.5546875" customWidth="true"/>
+    <col min="13" max="13" width="11.5546875" customWidth="true"/>
     <col min="15" max="15" width="36.44140625" customWidth="true"/>
   </cols>
   <sheetData>
@@ -19733,7 +20141,7 @@
         <v>848</v>
       </c>
       <c r="H2" s="0">
-        <v>0.0081850342654787404</v>
+        <v>0.008889416857156553</v>
       </c>
       <c r="I2" s="0">
         <v>3</v>
@@ -19742,13 +20150,13 @@
         <v>0</v>
       </c>
       <c r="K2" s="0">
-        <v>0.00272834475515958</v>
+        <v>0.0029631389523855178</v>
       </c>
       <c r="L2" s="0">
-        <v>0.023870732797348054</v>
+        <v>0.025930713454409178</v>
       </c>
       <c r="M2" s="0">
-        <v>0.9950070811308801</v>
+        <v>0.9943574819598584</v>
       </c>
       <c r="O2" s="0" t="s">
         <v>868</v>
@@ -19771,7 +20179,7 @@
         <v>849</v>
       </c>
       <c r="H3" s="0">
-        <v>92.923175202696996</v>
+        <v>92.902648919588501</v>
       </c>
       <c r="I3" s="0">
         <v>813</v>
@@ -19780,7 +20188,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="0">
-        <v>0.11429664846580197</v>
+        <v>0.11427140088510271</v>
       </c>
       <c r="L3" s="0"/>
       <c r="M3" s="0"/>
@@ -19790,22 +20198,22 @@
     </row>
     <row r="4">
       <c r="B4" s="0" t="s">
-        <v>1595</v>
+        <v>4259</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>1800</v>
+        <v>4266</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>2002</v>
+        <v>4273</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>2195</v>
+        <v>4280</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>850</v>
       </c>
       <c r="H4" s="0">
-        <v>92.931360236962476</v>
+        <v>92.911538336445659</v>
       </c>
       <c r="I4" s="0">
         <v>816</v>
@@ -19918,16 +20326,16 @@
         <v>859</v>
       </c>
       <c r="I11" s="0">
-        <v>-0.079058422086112565</v>
+        <v>-0.078790884655964191</v>
       </c>
       <c r="J11" s="0">
-        <v>0.0066249586217561607</v>
+        <v>0.006883032005597034</v>
       </c>
       <c r="K11" s="0">
-        <v>0.092308339329624886</v>
+        <v>0.092556948667158259</v>
       </c>
       <c r="L11" s="0">
-        <v>0.99722630733593265</v>
+        <v>0.99689199416926033</v>
       </c>
     </row>
     <row r="12">
@@ -19950,16 +20358,16 @@
         <v>860</v>
       </c>
       <c r="I12" s="0">
-        <v>-0.077311935902886236</v>
+        <v>-0.076952003172955516</v>
       </c>
       <c r="J12" s="0">
-        <v>0.0084766398575952806</v>
+        <v>0.0088270969220358708</v>
       </c>
       <c r="K12" s="0">
-        <v>0.094265215618076797</v>
+        <v>0.094606197017027258</v>
       </c>
       <c r="L12" s="0">
-        <v>0.99426504638935631</v>
+        <v>0.99353493481705168</v>
       </c>
     </row>
     <row r="13">
@@ -19982,16 +20390,16 @@
         <v>862</v>
       </c>
       <c r="I13" s="0">
-        <v>-0.080550744726213055</v>
+        <v>-0.080168350707049224</v>
       </c>
       <c r="J13" s="0">
-        <v>0.0054509501187069986</v>
+        <v>0.0058238449325895836</v>
       </c>
       <c r="K13" s="0">
-        <v>0.091452644963627053</v>
+        <v>0.091816040572228391</v>
       </c>
       <c r="L13" s="0">
-        <v>0.99846468723331794</v>
+        <v>0.99812956469902347</v>
       </c>
     </row>
     <row r="14">
@@ -20014,16 +20422,16 @@
         <v>860</v>
       </c>
       <c r="I14" s="0">
-        <v>-0.084040941301059879</v>
+        <v>-0.083939070462618739</v>
       </c>
       <c r="J14" s="0">
-        <v>0.0018516812358391199</v>
+        <v>0.0019440649164388368</v>
       </c>
       <c r="K14" s="0">
-        <v>0.087744303772738119</v>
+        <v>0.087827200295496413</v>
       </c>
       <c r="L14" s="0">
-        <v>0.99993905023043428</v>
+        <v>0.99992945036945535</v>
       </c>
     </row>
     <row r="15">
@@ -20046,16 +20454,16 @@
         <v>862</v>
       </c>
       <c r="I15" s="0">
-        <v>-0.08727949259931958</v>
+        <v>-0.087155160500089923</v>
       </c>
       <c r="J15" s="0">
-        <v>-0.001174008503049162</v>
+        <v>-0.0010591870730074504</v>
       </c>
       <c r="K15" s="0">
-        <v>0.084931475593221256</v>
+        <v>0.085036786354075022</v>
       </c>
       <c r="L15" s="0">
-        <v>0.99998456732714236</v>
+        <v>0.99998866126023112</v>
       </c>
     </row>
     <row r="16">
@@ -20078,16 +20486,16 @@
         <v>862</v>
       </c>
       <c r="I16" s="0">
-        <v>-0.089235853831850065</v>
+        <v>-0.089203893850927349</v>
       </c>
       <c r="J16" s="0">
-        <v>-0.003025689738888282</v>
+        <v>-0.0030032519894462872</v>
       </c>
       <c r="K16" s="0">
-        <v>0.083184474354073501</v>
+        <v>0.083197389872034774</v>
       </c>
       <c r="L16" s="0">
-        <v>0.99973752131071103</v>
+        <v>0.99974322099619595</v>
       </c>
     </row>
     <row r="17">
@@ -20216,16 +20624,16 @@
     </row>
     <row r="27">
       <c r="B27" s="0" t="s">
-        <v>1613</v>
+        <v>4260</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>1817</v>
+        <v>4267</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>2020</v>
+        <v>4274</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>2213</v>
+        <v>4281</v>
       </c>
     </row>
     <row r="28">
@@ -20568,16 +20976,16 @@
     </row>
     <row r="54">
       <c r="B54" s="0" t="s">
-        <v>1637</v>
+        <v>4261</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>1841</v>
+        <v>4268</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>2036</v>
+        <v>4275</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>2235</v>
+        <v>4282</v>
       </c>
     </row>
     <row r="55">
@@ -20666,16 +21074,16 @@
     </row>
     <row r="61">
       <c r="B61" s="0" t="s">
-        <v>1644</v>
+        <v>4262</v>
       </c>
       <c r="C61" s="0" t="s">
         <v>1848</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>1667</v>
+        <v>4276</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>2242</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="62">
@@ -22230,16 +22638,16 @@
     </row>
     <row r="189">
       <c r="B189" s="0" t="s">
-        <v>1745</v>
+        <v>4263</v>
       </c>
       <c r="C189" s="0" t="s">
-        <v>1947</v>
+        <v>4269</v>
       </c>
       <c r="D189" s="0" t="s">
-        <v>2142</v>
+        <v>4277</v>
       </c>
       <c r="E189" s="0" t="s">
-        <v>2329</v>
+        <v>4284</v>
       </c>
     </row>
     <row r="190">
@@ -22320,16 +22728,16 @@
     </row>
     <row r="196">
       <c r="B196" s="0" t="s">
-        <v>1751</v>
+        <v>4264</v>
       </c>
       <c r="C196" s="0" t="s">
-        <v>1953</v>
+        <v>4270</v>
       </c>
       <c r="D196" s="0" t="s">
-        <v>2148</v>
+        <v>4278</v>
       </c>
       <c r="E196" s="0" t="s">
-        <v>2334</v>
+        <v>4285</v>
       </c>
     </row>
     <row r="197">
@@ -22747,13 +23155,13 @@
         <v>1780</v>
       </c>
       <c r="C228" s="0" t="s">
-        <v>1981</v>
+        <v>4271</v>
       </c>
       <c r="D228" s="0" t="s">
         <v>2175</v>
       </c>
       <c r="E228" s="0" t="s">
-        <v>2360</v>
+        <v>4286</v>
       </c>
     </row>
     <row r="229">
@@ -23008,16 +23416,16 @@
     </row>
     <row r="248">
       <c r="B248" s="0" t="s">
-        <v>1797</v>
+        <v>4265</v>
       </c>
       <c r="C248" s="0" t="s">
-        <v>1999</v>
+        <v>4272</v>
       </c>
       <c r="D248" s="0" t="s">
-        <v>2192</v>
+        <v>4279</v>
       </c>
       <c r="E248" s="0" t="s">
-        <v>2377</v>
+        <v>4287</v>
       </c>
     </row>
     <row r="249">
@@ -23128,7 +23536,7 @@
         <v>848</v>
       </c>
       <c r="H2" s="0">
-        <v>5671.8511154255757</v>
+        <v>5614.0107095680096</v>
       </c>
       <c r="I2" s="0">
         <v>3</v>
@@ -23137,13 +23545,13 @@
         <v>0</v>
       </c>
       <c r="K2" s="0">
-        <v>1890.617038475192</v>
+        <v>1871.3369031893365</v>
       </c>
       <c r="L2" s="0">
-        <v>0.10383585244632065</v>
+        <v>0.10235756658429553</v>
       </c>
       <c r="M2" s="0">
-        <v>0.95782879556439449</v>
+        <v>0.9586720307699641</v>
       </c>
       <c r="O2" s="0" t="s">
         <v>868</v>
@@ -23166,7 +23574,7 @@
         <v>849</v>
       </c>
       <c r="H3" s="0">
-        <v>17625100.099121254</v>
+        <v>17697315.23263083</v>
       </c>
       <c r="I3" s="0">
         <v>968</v>
@@ -23175,7 +23583,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="0">
-        <v>18207.748036282286</v>
+        <v>18282.350446932676</v>
       </c>
       <c r="L3" s="0"/>
       <c r="M3" s="0"/>
@@ -23185,22 +23593,22 @@
     </row>
     <row r="4">
       <c r="B4" s="0" t="s">
-        <v>2380</v>
+        <v>4288</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>2577</v>
+        <v>4295</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>2775</v>
+        <v>4302</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>2967</v>
+        <v>4309</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>850</v>
       </c>
       <c r="H4" s="0">
-        <v>17630771.950236678</v>
+        <v>17702929.243340399</v>
       </c>
       <c r="I4" s="0">
         <v>971</v>
@@ -23329,16 +23737,16 @@
         <v>859</v>
       </c>
       <c r="I11" s="0">
-        <v>-32.370966614446544</v>
+        <v>-32.248845609915136</v>
       </c>
       <c r="J11" s="0">
-        <v>-0.98602500632748047</v>
+        <v>-0.79967313541328622</v>
       </c>
       <c r="K11" s="0">
-        <v>30.39891660179158</v>
+        <v>30.64949933908856</v>
       </c>
       <c r="L11" s="0">
-        <v>0.99981160843301808</v>
+        <v>0.99990003568501162</v>
       </c>
     </row>
     <row r="12">
@@ -23361,16 +23769,16 @@
         <v>860</v>
       </c>
       <c r="I12" s="0">
-        <v>-32.030952589939417</v>
+        <v>-31.809000626285883</v>
       </c>
       <c r="J12" s="0">
-        <v>-0.64601098182035344</v>
+        <v>-0.35982815178402916</v>
       </c>
       <c r="K12" s="0">
-        <v>30.738930626298714</v>
+        <v>31.089344322717825</v>
       </c>
       <c r="L12" s="0">
-        <v>0.99994694273744411</v>
+        <v>0.99999087757946215</v>
       </c>
     </row>
     <row r="13">
@@ -23393,16 +23801,16 @@
         <v>862</v>
       </c>
       <c r="I13" s="0">
-        <v>-26.459447433849462</v>
+        <v>-26.373507835080428</v>
       </c>
       <c r="J13" s="0">
-        <v>4.9908070626910899</v>
+        <v>5.1411111939641216</v>
       </c>
       <c r="K13" s="0">
-        <v>36.441061559231642</v>
+        <v>36.655730223008675</v>
       </c>
       <c r="L13" s="0">
-        <v>0.97712467467779063</v>
+        <v>0.97523457868539587</v>
       </c>
     </row>
     <row r="14">
@@ -23425,16 +23833,16 @@
         <v>860</v>
       </c>
       <c r="I14" s="0">
-        <v>-31.109175228350129</v>
+        <v>-31.073706621657053</v>
       </c>
       <c r="J14" s="0">
-        <v>0.34001402450712703</v>
+        <v>0.43984498362925706</v>
       </c>
       <c r="K14" s="0">
-        <v>31.789203277364383</v>
+        <v>31.953396588915567</v>
       </c>
       <c r="L14" s="0">
-        <v>0.99999230226850588</v>
+        <v>0.99998344573213105</v>
       </c>
     </row>
     <row r="15">
@@ -23457,16 +23865,16 @@
         <v>862</v>
       </c>
       <c r="I15" s="0">
-        <v>-25.537536920605163</v>
+        <v>-25.638080406295018</v>
       </c>
       <c r="J15" s="0">
-        <v>5.9768320690185703</v>
+        <v>5.9407843293774079</v>
       </c>
       <c r="K15" s="0">
-        <v>37.491201058642304</v>
+        <v>37.519649065049833</v>
       </c>
       <c r="L15" s="0">
-        <v>0.96196274776405766</v>
+        <v>0.96282314249969314</v>
       </c>
     </row>
     <row r="16">
@@ -23489,16 +23897,16 @@
         <v>862</v>
       </c>
       <c r="I16" s="0">
-        <v>-25.877550945112286</v>
+        <v>-26.077925389924268</v>
       </c>
       <c r="J16" s="0">
-        <v>5.6368180445114433</v>
+        <v>5.5009393457481508</v>
       </c>
       <c r="K16" s="0">
-        <v>37.151187034135177</v>
+        <v>37.079804081420569</v>
       </c>
       <c r="L16" s="0">
-        <v>0.96778230287565647</v>
+        <v>0.97011993761592974</v>
       </c>
     </row>
     <row r="17">
@@ -23643,16 +24051,16 @@
     </row>
     <row r="27">
       <c r="B27" s="0" t="s">
-        <v>2398</v>
+        <v>4289</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>2595</v>
+        <v>4296</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>2792</v>
+        <v>4303</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>2984</v>
+        <v>4310</v>
       </c>
     </row>
     <row r="28">
@@ -24011,16 +24419,16 @@
     </row>
     <row r="54">
       <c r="B54" s="0" t="s">
-        <v>2420</v>
+        <v>4290</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>2619</v>
+        <v>4297</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>2816</v>
+        <v>4304</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>3007</v>
+        <v>4311</v>
       </c>
     </row>
     <row r="55">
@@ -24109,16 +24517,16 @@
     </row>
     <row r="61">
       <c r="B61" s="0" t="s">
-        <v>2427</v>
+        <v>4291</v>
       </c>
       <c r="C61" s="0" t="s">
         <v>2626</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>2822</v>
+        <v>4305</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>3013</v>
+        <v>4312</v>
       </c>
     </row>
     <row r="62">
@@ -25863,16 +26271,16 @@
     </row>
     <row r="189">
       <c r="B189" s="0" t="s">
-        <v>2524</v>
+        <v>4292</v>
       </c>
       <c r="C189" s="0" t="s">
-        <v>2723</v>
+        <v>4298</v>
       </c>
       <c r="D189" s="0" t="s">
-        <v>2914</v>
+        <v>4306</v>
       </c>
       <c r="E189" s="0" t="s">
-        <v>3104</v>
+        <v>4313</v>
       </c>
     </row>
     <row r="190">
@@ -25961,16 +26369,16 @@
     </row>
     <row r="196">
       <c r="B196" s="0" t="s">
-        <v>2530</v>
+        <v>4293</v>
       </c>
       <c r="C196" s="0" t="s">
-        <v>2729</v>
+        <v>4299</v>
       </c>
       <c r="D196" s="0" t="s">
-        <v>2920</v>
+        <v>4307</v>
       </c>
       <c r="E196" s="0" t="s">
-        <v>3110</v>
+        <v>4314</v>
       </c>
     </row>
     <row r="197">
@@ -26412,13 +26820,13 @@
         <v>2556</v>
       </c>
       <c r="C228" s="0" t="s">
-        <v>2754</v>
+        <v>4300</v>
       </c>
       <c r="D228" s="0" t="s">
         <v>2948</v>
       </c>
       <c r="E228" s="0" t="s">
-        <v>3137</v>
+        <v>4315</v>
       </c>
     </row>
     <row r="229">
@@ -26689,16 +27097,16 @@
     </row>
     <row r="248">
       <c r="B248" s="0" t="s">
-        <v>2574</v>
+        <v>4294</v>
       </c>
       <c r="C248" s="0" t="s">
-        <v>2772</v>
+        <v>4301</v>
       </c>
       <c r="D248" s="0" t="s">
-        <v>2965</v>
+        <v>4308</v>
       </c>
       <c r="E248" s="0" t="s">
-        <v>3154</v>
+        <v>4316</v>
       </c>
     </row>
     <row r="249">
@@ -26760,7 +27168,7 @@
     <col min="7" max="7" width="6" customWidth="true"/>
     <col min="8" max="8" width="12.5546875" customWidth="true"/>
     <col min="9" max="9" width="13.21875" customWidth="true"/>
-    <col min="10" max="10" width="14.21875" customWidth="true"/>
+    <col min="10" max="10" width="15.21875" customWidth="true"/>
     <col min="11" max="11" width="12.5546875" customWidth="true"/>
     <col min="12" max="12" width="12.5546875" customWidth="true"/>
     <col min="13" max="13" width="12.5546875" customWidth="true"/>
@@ -26825,7 +27233,7 @@
         <v>848</v>
       </c>
       <c r="H2" s="0">
-        <v>1.100799859531763</v>
+        <v>1.0992063585398446</v>
       </c>
       <c r="I2" s="0">
         <v>3</v>
@@ -26834,13 +27242,13 @@
         <v>0</v>
       </c>
       <c r="K2" s="0">
-        <v>0.36693328651058765</v>
+        <v>0.36640211951328155</v>
       </c>
       <c r="L2" s="0">
-        <v>0.24777905691573249</v>
+        <v>0.24682202731993141</v>
       </c>
       <c r="M2" s="0">
-        <v>0.86294298123843938</v>
+        <v>0.86362363570482159</v>
       </c>
       <c r="O2" s="0" t="s">
         <v>868</v>
@@ -26863,7 +27271,7 @@
         <v>849</v>
       </c>
       <c r="H3" s="0">
-        <v>1433.5005781503412</v>
+        <v>1436.9756846260843</v>
       </c>
       <c r="I3" s="0">
         <v>968</v>
@@ -26872,7 +27280,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="0">
-        <v>1.4808890270148154</v>
+        <v>1.4844790130434755</v>
       </c>
       <c r="L3" s="0"/>
       <c r="M3" s="0"/>
@@ -26882,22 +27290,22 @@
     </row>
     <row r="4">
       <c r="B4" s="0" t="s">
-        <v>3157</v>
+        <v>4317</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>3299</v>
+        <v>4323</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>3419</v>
+        <v>4329</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>3517</v>
+        <v>4335</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>850</v>
       </c>
       <c r="H4" s="0">
-        <v>1434.6013780098729</v>
+        <v>1438.0748909846241</v>
       </c>
       <c r="I4" s="0">
         <v>971</v>
@@ -27026,16 +27434,16 @@
         <v>859</v>
       </c>
       <c r="I11" s="0">
-        <v>-0.22683433216575349</v>
+        <v>-0.22579565110213762</v>
       </c>
       <c r="J11" s="0">
-        <v>0.056210001532364551</v>
+        <v>0.057591554379426535</v>
       </c>
       <c r="K11" s="0">
-        <v>0.3392543352304826</v>
+        <v>0.34097875986099069</v>
       </c>
       <c r="L11" s="0">
-        <v>0.95669434278757981</v>
+        <v>0.95379977404629945</v>
       </c>
     </row>
     <row r="12">
@@ -27058,16 +27466,16 @@
         <v>860</v>
       </c>
       <c r="I12" s="0">
-        <v>-0.3186826061396702</v>
+        <v>-0.31747238071614592</v>
       </c>
       <c r="J12" s="0">
-        <v>-0.035638272441552044</v>
+        <v>-0.034085175234581655</v>
       </c>
       <c r="K12" s="0">
-        <v>0.24740606125656611</v>
+        <v>0.24930203024698261</v>
       </c>
       <c r="L12" s="0">
-        <v>0.98830953611783456</v>
+        <v>0.98977461556054158</v>
       </c>
     </row>
     <row r="13">
@@ -27090,16 +27498,16 @@
         <v>862</v>
       </c>
       <c r="I13" s="0">
-        <v>-0.29477281572457831</v>
+        <v>-0.29366881743430051</v>
       </c>
       <c r="J13" s="0">
-        <v>-0.011139459328378232</v>
+        <v>-0.0096918757294608415</v>
       </c>
       <c r="K13" s="0">
-        <v>0.27249389706782184</v>
+        <v>0.27428506597537883</v>
       </c>
       <c r="L13" s="0">
-        <v>0.99963247978474079</v>
+        <v>0.99975859678010126</v>
       </c>
     </row>
     <row r="14">
@@ -27122,16 +27530,16 @@
         <v>860</v>
       </c>
       <c r="I14" s="0">
-        <v>-0.3754720234958287</v>
+        <v>-0.37564405280706809</v>
       </c>
       <c r="J14" s="0">
-        <v>-0.091848273973916594</v>
+        <v>-0.09167672961400819</v>
       </c>
       <c r="K14" s="0">
-        <v>0.19177547554799551</v>
+        <v>0.19229059357905171</v>
       </c>
       <c r="L14" s="0">
-        <v>0.83929897193162994</v>
+        <v>0.8405371713694465</v>
       </c>
     </row>
     <row r="15">
@@ -27154,16 +27562,16 @@
         <v>862</v>
       </c>
       <c r="I15" s="0">
-        <v>-0.35156103225576979</v>
+        <v>-0.35183928724561081</v>
       </c>
       <c r="J15" s="0">
-        <v>-0.067349460860742782</v>
+        <v>-0.067283430108887377</v>
       </c>
       <c r="K15" s="0">
-        <v>0.21686211053428422</v>
+        <v>0.21727242702783606</v>
       </c>
       <c r="L15" s="0">
-        <v>0.9293302905160008</v>
+        <v>0.92975197826703249</v>
       </c>
     </row>
     <row r="16">
@@ -27186,16 +27594,16 @@
         <v>862</v>
       </c>
       <c r="I16" s="0">
-        <v>-0.25971275828185308</v>
+        <v>-0.26016255763160251</v>
       </c>
       <c r="J16" s="0">
-        <v>0.024498813113173812</v>
+        <v>0.024393299505120813</v>
       </c>
       <c r="K16" s="0">
-        <v>0.30871038450820071</v>
+        <v>0.30894915664184414</v>
       </c>
       <c r="L16" s="0">
-        <v>0.99617040278761193</v>
+        <v>0.9962326172484669</v>
       </c>
     </row>
     <row r="17">
@@ -27340,16 +27748,16 @@
     </row>
     <row r="27">
       <c r="B27" s="0" t="s">
-        <v>3173</v>
+        <v>4318</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>3203</v>
+        <v>4324</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>3428</v>
+        <v>4330</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>3529</v>
+        <v>4336</v>
       </c>
     </row>
     <row r="28">
@@ -27708,16 +28116,16 @@
     </row>
     <row r="54">
       <c r="B54" s="0" t="s">
-        <v>3193</v>
+        <v>4319</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>3255</v>
+        <v>4325</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>3442</v>
+        <v>4331</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>3542</v>
+        <v>4337</v>
       </c>
     </row>
     <row r="55">
@@ -27806,16 +28214,16 @@
     </row>
     <row r="61">
       <c r="B61" s="0" t="s">
-        <v>1208</v>
+        <v>1547</v>
       </c>
       <c r="C61" s="0" t="s">
         <v>3330</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>3254</v>
+        <v>4332</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>3546</v>
+        <v>4338</v>
       </c>
     </row>
     <row r="62">
@@ -29560,16 +29968,16 @@
     </row>
     <row r="189">
       <c r="B189" s="0" t="s">
-        <v>3261</v>
+        <v>4320</v>
       </c>
       <c r="C189" s="0" t="s">
-        <v>3380</v>
+        <v>4326</v>
       </c>
       <c r="D189" s="0" t="s">
-        <v>3487</v>
+        <v>4333</v>
       </c>
       <c r="E189" s="0" t="s">
-        <v>3587</v>
+        <v>4339</v>
       </c>
     </row>
     <row r="190">
@@ -29658,16 +30066,16 @@
     </row>
     <row r="196">
       <c r="B196" s="0" t="s">
-        <v>1253</v>
+        <v>4321</v>
       </c>
       <c r="C196" s="0" t="s">
-        <v>3383</v>
+        <v>4327</v>
       </c>
       <c r="D196" s="0" t="s">
-        <v>3492</v>
+        <v>4334</v>
       </c>
       <c r="E196" s="0" t="s">
-        <v>3159</v>
+        <v>4340</v>
       </c>
     </row>
     <row r="197">
@@ -30109,13 +30517,13 @@
         <v>3174</v>
       </c>
       <c r="C228" s="0" t="s">
-        <v>3404</v>
+        <v>111</v>
       </c>
       <c r="D228" s="0" t="s">
         <v>3506</v>
       </c>
       <c r="E228" s="0" t="s">
-        <v>3605</v>
+        <v>4341</v>
       </c>
     </row>
     <row r="229">
@@ -30386,16 +30794,16 @@
     </row>
     <row r="248">
       <c r="B248" s="0" t="s">
-        <v>3296</v>
+        <v>4322</v>
       </c>
       <c r="C248" s="0" t="s">
-        <v>3416</v>
+        <v>4328</v>
       </c>
       <c r="D248" s="0" t="s">
-        <v>3515</v>
+        <v>1745</v>
       </c>
       <c r="E248" s="0" t="s">
-        <v>3614</v>
+        <v>4342</v>
       </c>
     </row>
     <row r="249">

</xml_diff>